<commit_message>
Updated readme file and added traits excel sheet for review.
</commit_message>
<xml_diff>
--- a/server/traits.xlsx
+++ b/server/traits.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>Trait</t>
   </si>
@@ -31,13 +31,133 @@
     <t>Activation Rate</t>
   </si>
   <si>
-    <t>$__parent</t>
-  </si>
-  <si>
-    <t>$__path</t>
-  </si>
-  <si>
-    <t>$__schemaType</t>
+    <t>TFT16_Brawler</t>
+  </si>
+  <si>
+    <t>TFT16_Defender</t>
+  </si>
+  <si>
+    <t>TFT16_Emperor</t>
+  </si>
+  <si>
+    <t>TFT16_Invoker</t>
+  </si>
+  <si>
+    <t>TFT16_Juggernaut</t>
+  </si>
+  <si>
+    <t>TFT16_KindredUnique</t>
+  </si>
+  <si>
+    <t>TFT16_Magus</t>
+  </si>
+  <si>
+    <t>TFT16_Noxus</t>
+  </si>
+  <si>
+    <t>TFT16_Rapidfire</t>
+  </si>
+  <si>
+    <t>TFT16_Shurima</t>
+  </si>
+  <si>
+    <t>TFT16_Sorcerer</t>
+  </si>
+  <si>
+    <t>TFT16_Vanquisher</t>
+  </si>
+  <si>
+    <t>TFT16_Bilgewater</t>
+  </si>
+  <si>
+    <t>TFT16_Explorer</t>
+  </si>
+  <si>
+    <t>TFT16_Freljord</t>
+  </si>
+  <si>
+    <t>TFT16_Gunslinger</t>
+  </si>
+  <si>
+    <t>TFT16_Ionia</t>
+  </si>
+  <si>
+    <t>TFT16_Slayer</t>
+  </si>
+  <si>
+    <t>TFT16_Soulbound</t>
+  </si>
+  <si>
+    <t>TFT16_Yordle</t>
+  </si>
+  <si>
+    <t>TFT16_Zaun</t>
+  </si>
+  <si>
+    <t>TFT15_Bastion</t>
+  </si>
+  <si>
+    <t>TFT15_Destroyer</t>
+  </si>
+  <si>
+    <t>TFT15_Duelist</t>
+  </si>
+  <si>
+    <t>TFT15_Edgelord</t>
+  </si>
+  <si>
+    <t>TFT15_Juggernaut</t>
+  </si>
+  <si>
+    <t>TFT15_Luchador</t>
+  </si>
+  <si>
+    <t>TFT15_SoulFighter</t>
+  </si>
+  <si>
+    <t>TFT15_Spellslinger</t>
+  </si>
+  <si>
+    <t>TFT15_GemForce</t>
+  </si>
+  <si>
+    <t>TFT15_Heavyweight</t>
+  </si>
+  <si>
+    <t>TFT15_Prodigy</t>
+  </si>
+  <si>
+    <t>TFT15_Protector</t>
+  </si>
+  <si>
+    <t>TFT15_Sniper</t>
+  </si>
+  <si>
+    <t>TFT15_StarGuardian</t>
+  </si>
+  <si>
+    <t>TFT15_BattleAcademia</t>
+  </si>
+  <si>
+    <t>TFT15_Empyrean</t>
+  </si>
+  <si>
+    <t>TFT15_MonsterTrainer</t>
+  </si>
+  <si>
+    <t>TFT15_OldMentor</t>
+  </si>
+  <si>
+    <t>TFT15_SentaiRanger</t>
+  </si>
+  <si>
+    <t>TFT15_Strategist</t>
+  </si>
+  <si>
+    <t>TFT15_SupremeCells</t>
+  </si>
+  <si>
+    <t>TFT15_TheCrew</t>
   </si>
 </sst>
 </file>
@@ -414,7 +534,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -437,25 +557,864 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
       <c r="D2">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>4.2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0.5</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>4</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
+        <v>4</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>4</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23">
+        <v>5</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>0.6</v>
+      </c>
+      <c r="E23">
+        <v>3</v>
+      </c>
+      <c r="F23">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24">
+        <v>6</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>1.1666666666666667</v>
+      </c>
+      <c r="F24">
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25">
+        <v>4</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>0.25</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26">
+        <v>6</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="E26">
+        <v>1.6666666666666667</v>
+      </c>
+      <c r="F26">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27">
+        <v>4</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>0.25</v>
+      </c>
+      <c r="E27">
+        <v>5.5</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28">
+        <v>3</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29">
+        <v>4</v>
+      </c>
+      <c r="C29">
+        <v>0</v>
+      </c>
+      <c r="D29">
+        <v>0.25</v>
+      </c>
+      <c r="E29">
+        <v>3.75</v>
+      </c>
+      <c r="F29">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30">
+        <v>8</v>
+      </c>
+      <c r="C30">
+        <v>0</v>
+      </c>
+      <c r="D30">
+        <v>0.25</v>
+      </c>
+      <c r="E30">
+        <v>3</v>
+      </c>
+      <c r="F30">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31">
+        <v>5</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>37</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>0.5</v>
+      </c>
+      <c r="E33">
+        <v>2</v>
+      </c>
+      <c r="F33">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>38</v>
+      </c>
+      <c r="B34">
+        <v>4</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+      <c r="D34">
+        <v>0.75</v>
+      </c>
+      <c r="E34">
+        <v>2.25</v>
+      </c>
+      <c r="F34">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>39</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>40</v>
+      </c>
+      <c r="B36">
+        <v>4</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>0.5</v>
+      </c>
+      <c r="E36">
+        <v>1.5</v>
+      </c>
+      <c r="F36">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>41</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>42</v>
+      </c>
+      <c r="B38">
+        <v>2</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>43</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39">
+        <v>0</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>3.5</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B40">
+        <v>3</v>
+      </c>
+      <c r="C40">
+        <v>0</v>
+      </c>
+      <c r="D40">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="E40">
+        <v>4.666666666666667</v>
+      </c>
+      <c r="F40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>45</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41">
+        <v>0</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>3.5</v>
+      </c>
+      <c r="F41">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>46</v>
+      </c>
+      <c r="B42">
+        <v>3</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="E42">
+        <v>2.3333333333333335</v>
+      </c>
+      <c r="F42">
+        <v>0.6666666666666666</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44">
+        <v>2</v>
+      </c>
+      <c r="C44">
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>